<commit_message>
Rebuild capacity model independently, extend report through Design Alternatives
- Rebuild all discretionary workbook assumptions (storage, personnel, parking,
  evaluation scores, nesting/packaging) with independent values
- Add Space Requirements and Design Alternatives sections to 417.docx
- Add nine workstation subsections (sheet/hinge, finishing, heat treat,
  sandblast, powder coat, assembly/packaging) with market-example equipment
- Remove named benchmark references from report text
- Add ChatGPT Section 8 draft package and figure exports for reference
- Export refreshed 417.pdf

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/05_Working/5.1_Capacity_Model/417.xlsx
+++ b/05_Working/5.1_Capacity_Model/417.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\NB444144\Downloads\INGB 417 EXAM ASSIGNMENT\INGB 417 EXAM ASSIGNMENT\05_Working\5.1_Capacity_Model\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6c73f9ad2dbf6c5f/INGB 417 EXAM ASSIGNMENT/05_Working/5.1_Capacity_Model/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{533E76B1-A49F-43DF-BAEE-8B6B7AFD13BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="88" documentId="13_ncr:1_{533E76B1-A49F-43DF-BAEE-8B6B7AFD13BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D3AC88CA-F785-4994-A153-BACA73751B4E}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="500" firstSheet="12" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" firstSheet="12" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Inputs" sheetId="1" r:id="rId1"/>
@@ -2524,6 +2524,10 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -2704,24 +2708,24 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E60"/>
-  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="30" customWidth="1"/>
     <col min="3" max="4" width="12" customWidth="1"/>
     <col min="5" max="5" width="46" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" ht="16.8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>487</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B4" s="3" t="s">
         <v>1</v>
       </c>
@@ -2735,7 +2739,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B5" s="4" t="s">
         <v>5</v>
       </c>
@@ -2749,7 +2753,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B6" s="4" t="s">
         <v>8</v>
       </c>
@@ -2763,7 +2767,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B7" s="4" t="s">
         <v>10</v>
       </c>
@@ -2778,7 +2782,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B8" s="4" t="s">
         <v>13</v>
       </c>
@@ -2792,7 +2796,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B9" s="4" t="s">
         <v>16</v>
       </c>
@@ -2806,7 +2810,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B10" s="4" t="s">
         <v>18</v>
       </c>
@@ -2821,7 +2825,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B11" s="4" t="s">
         <v>21</v>
       </c>
@@ -2835,7 +2839,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B12" s="4" t="s">
         <v>24</v>
       </c>
@@ -2850,7 +2854,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B13" s="4" t="s">
         <v>26</v>
       </c>
@@ -2865,7 +2869,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B14" s="4" t="s">
         <v>29</v>
       </c>
@@ -2879,7 +2883,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B15" s="4" t="s">
         <v>31</v>
       </c>
@@ -2894,7 +2898,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B16" s="4" t="s">
         <v>33</v>
       </c>
@@ -2908,7 +2912,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B17" s="4" t="s">
         <v>36</v>
       </c>
@@ -2922,7 +2926,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B18" s="4" t="s">
         <v>39</v>
       </c>
@@ -2936,12 +2940,12 @@
         <v>40</v>
       </c>
     </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B19" s="4" t="s">
         <v>41</v>
       </c>
       <c r="C19" s="8">
-        <v>6</v>
+        <v>6.5</v>
       </c>
       <c r="D19" s="6" t="s">
         <v>42</v>
@@ -2950,7 +2954,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B20" s="4" t="s">
         <v>44</v>
       </c>
@@ -2964,13 +2968,13 @@
         <v>45</v>
       </c>
     </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B21" s="4" t="s">
         <v>46</v>
       </c>
       <c r="C21" s="6">
         <f>FLOOR(C19/C20,1)</f>
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="D21" s="6" t="s">
         <v>47</v>
@@ -2979,7 +2983,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B22" s="4" t="s">
         <v>49</v>
       </c>
@@ -2993,7 +2997,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B23" s="4" t="s">
         <v>51</v>
       </c>
@@ -3007,7 +3011,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B24" s="4" t="s">
         <v>53</v>
       </c>
@@ -3021,12 +3025,12 @@
         <v>52</v>
       </c>
     </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B25" s="4" t="s">
         <v>54</v>
       </c>
       <c r="C25" s="8">
-        <v>0.75</v>
+        <v>0.8</v>
       </c>
       <c r="D25" s="6" t="s">
         <v>22</v>
@@ -3035,7 +3039,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="26" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B26" s="4" t="s">
         <v>56</v>
       </c>
@@ -3049,7 +3053,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="27" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B27" s="4" t="s">
         <v>58</v>
       </c>
@@ -3063,7 +3067,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="28" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B28" s="4" t="s">
         <v>60</v>
       </c>
@@ -3077,7 +3081,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="29" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B29" s="4" t="s">
         <v>61</v>
       </c>
@@ -3091,7 +3095,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="30" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B30" s="4" t="s">
         <v>62</v>
       </c>
@@ -3105,7 +3109,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="31" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B31" s="4" t="s">
         <v>64</v>
       </c>
@@ -3119,7 +3123,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="32" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B32" s="4" t="s">
         <v>66</v>
       </c>
@@ -3133,12 +3137,12 @@
         <v>67</v>
       </c>
     </row>
-    <row r="33" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B33" s="4" t="s">
         <v>68</v>
       </c>
       <c r="C33" s="8">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D33" s="6" t="s">
         <v>69</v>
@@ -3147,12 +3151,12 @@
         <v>55</v>
       </c>
     </row>
-    <row r="34" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B34" s="4" t="s">
         <v>70</v>
       </c>
       <c r="C34" s="8">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="D34" s="6" t="s">
         <v>71</v>
@@ -3161,13 +3165,13 @@
         <v>55</v>
       </c>
     </row>
-    <row r="35" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B35" s="4" t="s">
         <v>72</v>
       </c>
       <c r="C35" s="6">
         <f>C33*C34</f>
-        <v>400</v>
+        <v>360</v>
       </c>
       <c r="D35" s="6" t="s">
         <v>69</v>
@@ -3176,7 +3180,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="36" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="36" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B36" s="4" t="s">
         <v>74</v>
       </c>
@@ -3190,7 +3194,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="37" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="37" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B37" s="4" t="s">
         <v>76</v>
       </c>
@@ -3204,7 +3208,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="38" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="38" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B38" s="4" t="s">
         <v>77</v>
       </c>
@@ -3217,12 +3221,12 @@
       </c>
       <c r="E38" s="7"/>
     </row>
-    <row r="39" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="39" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B39" s="4" t="s">
         <v>79</v>
       </c>
       <c r="C39" s="8">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D39" s="6" t="s">
         <v>37</v>
@@ -3231,12 +3235,12 @@
         <v>55</v>
       </c>
     </row>
-    <row r="40" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="40" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B40" s="4" t="s">
         <v>80</v>
       </c>
       <c r="C40" s="8">
-        <v>250</v>
+        <v>200</v>
       </c>
       <c r="D40" s="6" t="s">
         <v>81</v>
@@ -3245,12 +3249,12 @@
         <v>55</v>
       </c>
     </row>
-    <row r="41" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="41" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B41" s="4" t="s">
         <v>82</v>
       </c>
       <c r="C41" s="8">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D41" s="6" t="s">
         <v>78</v>
@@ -3259,12 +3263,12 @@
         <v>83</v>
       </c>
     </row>
-    <row r="42" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="42" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B42" s="4" t="s">
         <v>84</v>
       </c>
       <c r="C42" s="8">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="D42" s="6" t="s">
         <v>85</v>
@@ -3273,12 +3277,12 @@
         <v>55</v>
       </c>
     </row>
-    <row r="43" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="43" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B43" s="4" t="s">
         <v>86</v>
       </c>
       <c r="C43" s="8">
-        <v>1.6</v>
+        <v>1.5</v>
       </c>
       <c r="D43" s="6" t="s">
         <v>37</v>
@@ -3287,7 +3291,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="44" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="44" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B44" s="4" t="s">
         <v>88</v>
       </c>
@@ -3301,7 +3305,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="45" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="45" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B45" s="4" t="s">
         <v>91</v>
       </c>
@@ -3315,7 +3319,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="46" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="46" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B46" s="4" t="s">
         <v>94</v>
       </c>
@@ -3329,12 +3333,12 @@
         <v>96</v>
       </c>
     </row>
-    <row r="47" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="47" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B47" s="4" t="s">
         <v>97</v>
       </c>
       <c r="C47" s="8">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D47" s="6" t="s">
         <v>78</v>
@@ -3343,12 +3347,12 @@
         <v>98</v>
       </c>
     </row>
-    <row r="48" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="48" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B48" s="4" t="s">
         <v>99</v>
       </c>
       <c r="C48" s="8">
-        <v>0.3</v>
+        <v>0.25</v>
       </c>
       <c r="D48" s="6" t="s">
         <v>22</v>
@@ -3357,7 +3361,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="49" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="49" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B49" s="4" t="s">
         <v>100</v>
       </c>
@@ -3371,12 +3375,12 @@
         <v>101</v>
       </c>
     </row>
-    <row r="50" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="50" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B50" s="4" t="s">
         <v>102</v>
       </c>
       <c r="C50" s="8">
-        <v>120</v>
+        <v>135</v>
       </c>
       <c r="D50" s="6" t="s">
         <v>78</v>
@@ -3385,12 +3389,12 @@
         <v>103</v>
       </c>
     </row>
-    <row r="51" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="51" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B51" s="4" t="s">
         <v>104</v>
       </c>
       <c r="C51" s="8">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="D51" s="6" t="s">
         <v>78</v>
@@ -3399,12 +3403,12 @@
         <v>103</v>
       </c>
     </row>
-    <row r="52" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="52" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B52" s="4" t="s">
         <v>105</v>
       </c>
       <c r="C52" s="8">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="D52" s="6" t="s">
         <v>78</v>
@@ -3413,12 +3417,12 @@
         <v>55</v>
       </c>
     </row>
-    <row r="53" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="53" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B53" s="4" t="s">
         <v>106</v>
       </c>
       <c r="C53" s="8">
-        <v>250</v>
+        <v>220</v>
       </c>
       <c r="D53" s="6" t="s">
         <v>78</v>
@@ -3427,12 +3431,12 @@
         <v>107</v>
       </c>
     </row>
-    <row r="54" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="54" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B54" s="4" t="s">
         <v>108</v>
       </c>
       <c r="C54" s="8">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D54" s="6" t="s">
         <v>78</v>
@@ -3441,12 +3445,12 @@
         <v>55</v>
       </c>
     </row>
-    <row r="55" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="55" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B55" s="4" t="s">
         <v>109</v>
       </c>
       <c r="C55" s="8">
-        <v>4</v>
+        <v>3.5</v>
       </c>
       <c r="D55" s="6" t="s">
         <v>78</v>
@@ -3455,7 +3459,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="56" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="56" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B56" s="4" t="s">
         <v>111</v>
       </c>
@@ -3469,12 +3473,12 @@
         <v>112</v>
       </c>
     </row>
-    <row r="57" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="57" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B57" s="4" t="s">
         <v>113</v>
       </c>
       <c r="C57" s="8">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D57" s="6" t="s">
         <v>114</v>
@@ -3483,12 +3487,12 @@
         <v>55</v>
       </c>
     </row>
-    <row r="58" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="58" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B58" s="4" t="s">
         <v>115</v>
       </c>
       <c r="C58" s="8">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="D58" s="6" t="s">
         <v>78</v>
@@ -3497,12 +3501,12 @@
         <v>116</v>
       </c>
     </row>
-    <row r="59" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="59" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B59" s="4" t="s">
         <v>117</v>
       </c>
       <c r="C59" s="8">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D59" s="6" t="s">
         <v>114</v>
@@ -3511,12 +3515,12 @@
         <v>118</v>
       </c>
     </row>
-    <row r="60" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="60" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B60" s="4" t="s">
         <v>119</v>
       </c>
       <c r="C60" s="8">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="D60" s="6" t="s">
         <v>78</v>
@@ -3534,26 +3538,26 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:C19"/>
-  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="37.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.90625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="28.6328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="37.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="28.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="17" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A1" s="27" t="s">
         <v>288</v>
       </c>
       <c r="B1" s="27"/>
       <c r="C1" s="27"/>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="25"/>
       <c r="B2" s="25"/>
       <c r="C2" s="25"/>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="28" t="s">
         <v>289</v>
       </c>
@@ -3564,178 +3568,178 @@
         <v>123</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="25" t="s">
         <v>290</v>
       </c>
       <c r="B4" s="25">
         <f>Capacity!M18*Inputs!$C$47</f>
-        <v>204</v>
+        <v>238</v>
       </c>
       <c r="C4" s="26" t="s">
         <v>291</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="25" t="s">
         <v>292</v>
       </c>
       <c r="B5" s="25">
         <f>Inputs!$C$50</f>
-        <v>120</v>
+        <v>135</v>
       </c>
       <c r="C5" s="26" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="25" t="s">
         <v>293</v>
       </c>
       <c r="B6" s="25">
         <f>Inputs!$C$51</f>
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="C6" s="26" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="25" t="s">
         <v>294</v>
       </c>
       <c r="B7" s="25">
         <f>Storage_3D!D4+Storage_3D!D5+Storage_3D!D7+Storage_3D!D8</f>
-        <v>92.240000000000009</v>
+        <v>80.474999999999994</v>
       </c>
       <c r="C7" s="26" t="s">
         <v>295</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="25" t="s">
         <v>296</v>
       </c>
       <c r="B8" s="25">
         <f>Storage_3D!D6</f>
-        <v>59.519999999999996</v>
+        <v>46.8</v>
       </c>
       <c r="C8" s="26" t="s">
         <v>295</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="25" t="s">
         <v>297</v>
       </c>
       <c r="B9" s="25">
         <f>Inputs!$C$53</f>
-        <v>250</v>
+        <v>220</v>
       </c>
       <c r="C9" s="26" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" s="25" t="s">
         <v>298</v>
       </c>
       <c r="B10" s="25">
         <f>(Personnel!B18-Capacity!O18)*Inputs!$C$54</f>
-        <v>260</v>
+        <v>216</v>
       </c>
       <c r="C10" s="26" t="s">
         <v>299</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="35" t="s">
         <v>300</v>
       </c>
       <c r="B11" s="35">
         <f>Personnel!B18*Inputs!$C$55</f>
-        <v>240</v>
+        <v>203</v>
       </c>
       <c r="C11" s="38" t="s">
         <v>301</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" s="40" t="s">
         <v>302</v>
       </c>
       <c r="B12" s="40">
         <f>SUM(B4:B11)</f>
-        <v>1305.76</v>
+        <v>1209.2750000000001</v>
       </c>
       <c r="C12" s="40"/>
     </row>
-    <row r="13" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" s="44" t="s">
         <v>303</v>
       </c>
       <c r="B13" s="44">
         <f>B12*Inputs!$C$48</f>
-        <v>391.72800000000001</v>
+        <v>302.31875000000002</v>
       </c>
       <c r="C13" s="45" t="s">
         <v>304</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" s="40" t="s">
         <v>305</v>
       </c>
       <c r="B14" s="40">
         <f>B12+B13</f>
-        <v>1697.4880000000001</v>
+        <v>1511.59375</v>
       </c>
       <c r="C14" s="40"/>
     </row>
-    <row r="15" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="44" t="s">
         <v>306</v>
       </c>
       <c r="B15" s="44">
         <f>ROUND(B14*Inputs!$C$49,0)</f>
-        <v>170</v>
+        <v>151</v>
       </c>
       <c r="C15" s="44"/>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" s="46" t="s">
         <v>307</v>
       </c>
       <c r="B16" s="46">
         <f>ROUND(B14+B15,0)</f>
-        <v>1867</v>
+        <v>1663</v>
       </c>
       <c r="C16" s="46"/>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" s="39"/>
       <c r="B17" s="39"/>
       <c r="C17" s="39"/>
     </row>
-    <row r="18" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A18" s="35" t="s">
         <v>308</v>
       </c>
       <c r="B18" s="35">
         <f>Parking!B10</f>
-        <v>2110</v>
+        <v>2198</v>
       </c>
       <c r="C18" s="38" t="s">
         <v>309</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" s="46" t="s">
         <v>310</v>
       </c>
       <c r="B19" s="46">
         <f>ROUND(B16+B18,0)</f>
-        <v>3977</v>
+        <v>3861</v>
       </c>
       <c r="C19" s="46"/>
     </row>
@@ -3748,7 +3752,7 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:F15"/>
-  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
     <col min="2" max="2" width="34" customWidth="1"/>
@@ -3758,12 +3762,12 @@
     <col min="6" max="6" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" ht="16.8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>311</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>312</v>
       </c>
@@ -3783,7 +3787,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
         <v>157</v>
       </c>
@@ -3803,7 +3807,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>323</v>
       </c>
@@ -3823,7 +3827,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>326</v>
       </c>
@@ -3843,7 +3847,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>329</v>
       </c>
@@ -3863,7 +3867,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
         <v>331</v>
       </c>
@@ -3883,7 +3887,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
         <v>334</v>
       </c>
@@ -3903,7 +3907,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
         <v>336</v>
       </c>
@@ -3923,7 +3927,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
         <v>339</v>
       </c>
@@ -3943,7 +3947,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
         <v>342</v>
       </c>
@@ -3963,7 +3967,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
         <v>345</v>
       </c>
@@ -3983,7 +3987,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>349</v>
       </c>
@@ -3997,19 +4001,19 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <dimension ref="A1:H17"/>
-  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="40.6328125" customWidth="1"/>
-    <col min="2" max="2" width="10.6328125" customWidth="1"/>
-    <col min="3" max="8" width="18.6328125" customWidth="1"/>
+    <col min="1" max="1" width="40.6640625" customWidth="1"/>
+    <col min="2" max="2" width="10.6640625" customWidth="1"/>
+    <col min="3" max="8" width="18.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" ht="16.8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>350</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="42" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>351</v>
       </c>
@@ -4035,7 +4039,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="6" t="s">
         <v>356</v>
       </c>
@@ -4064,7 +4068,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="6" t="s">
         <v>357</v>
       </c>
@@ -4075,7 +4079,7 @@
         <v>5</v>
       </c>
       <c r="D5" s="5">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E5" s="5">
         <v>4</v>
@@ -4086,14 +4090,14 @@
       </c>
       <c r="G5" s="6">
         <f t="shared" si="1"/>
-        <v>0.8</v>
+        <v>0.60000000000000009</v>
       </c>
       <c r="H5" s="6">
         <f t="shared" si="2"/>
         <v>0.8</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="6" t="s">
         <v>358</v>
       </c>
@@ -4104,7 +4108,7 @@
         <v>3</v>
       </c>
       <c r="D6" s="5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E6" s="5">
         <v>5</v>
@@ -4115,14 +4119,14 @@
       </c>
       <c r="G6" s="6">
         <f t="shared" si="1"/>
-        <v>0.44999999999999996</v>
+        <v>0.3</v>
       </c>
       <c r="H6" s="6">
         <f t="shared" si="2"/>
         <v>0.75</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="6" t="s">
         <v>359</v>
       </c>
@@ -4130,28 +4134,28 @@
         <v>0.15</v>
       </c>
       <c r="C7" s="5">
+        <v>3</v>
+      </c>
+      <c r="D7" s="5">
         <v>4</v>
       </c>
-      <c r="D7" s="5">
-        <v>5</v>
-      </c>
       <c r="E7" s="5">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F7" s="6">
         <f t="shared" si="0"/>
-        <v>0.6</v>
+        <v>0.44999999999999996</v>
       </c>
       <c r="G7" s="6">
         <f t="shared" si="1"/>
-        <v>0.75</v>
+        <v>0.6</v>
       </c>
       <c r="H7" s="6">
         <f t="shared" si="2"/>
-        <v>0.6</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+        <v>0.44999999999999996</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="6" t="s">
         <v>360</v>
       </c>
@@ -4159,7 +4163,7 @@
         <v>0.1</v>
       </c>
       <c r="C8" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D8" s="5">
         <v>3</v>
@@ -4169,7 +4173,7 @@
       </c>
       <c r="F8" s="6">
         <f t="shared" si="0"/>
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="G8" s="6">
         <f t="shared" si="1"/>
@@ -4180,7 +4184,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" s="6" t="s">
         <v>361</v>
       </c>
@@ -4188,7 +4192,7 @@
         <v>0.1</v>
       </c>
       <c r="C9" s="5">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D9" s="5">
         <v>2</v>
@@ -4198,7 +4202,7 @@
       </c>
       <c r="F9" s="6">
         <f t="shared" si="0"/>
-        <v>0.4</v>
+        <v>0.30000000000000004</v>
       </c>
       <c r="G9" s="6">
         <f t="shared" si="1"/>
@@ -4209,7 +4213,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" s="6" t="s">
         <v>362</v>
       </c>
@@ -4238,7 +4242,7 @@
         <v>0.30000000000000004</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" s="9" t="s">
         <v>363</v>
       </c>
@@ -4251,38 +4255,38 @@
       <c r="E11" s="10"/>
       <c r="F11" s="9">
         <f>SUM(F4:F10)</f>
-        <v>4.45</v>
+        <v>4.1000000000000005</v>
       </c>
       <c r="G11" s="9">
         <f>SUM(G4:G10)</f>
-        <v>3.9</v>
+        <v>3.4</v>
       </c>
       <c r="H11" s="9">
         <f>SUM(H4:H10)</f>
-        <v>4.3499999999999996</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+        <v>4.2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>444</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>445</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>446</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>447</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>448</v>
       </c>
@@ -4296,18 +4300,18 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{909F8702-1A62-4461-BF14-5A3044C31F17}">
   <dimension ref="A1:G15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="44.08984375" customWidth="1"/>
-    <col min="2" max="2" width="28.54296875" customWidth="1"/>
-    <col min="3" max="3" width="44.08984375" customWidth="1"/>
-    <col min="4" max="4" width="59.6328125" customWidth="1"/>
-    <col min="5" max="5" width="31.08984375" customWidth="1"/>
-    <col min="6" max="6" width="18.08984375" customWidth="1"/>
-    <col min="7" max="7" width="38.90625" customWidth="1"/>
+    <col min="1" max="1" width="44.109375" customWidth="1"/>
+    <col min="2" max="2" width="28.5546875" customWidth="1"/>
+    <col min="3" max="3" width="44.109375" customWidth="1"/>
+    <col min="4" max="4" width="59.6640625" customWidth="1"/>
+    <col min="5" max="5" width="31.109375" customWidth="1"/>
+    <col min="6" max="6" width="18.109375" customWidth="1"/>
+    <col min="7" max="7" width="38.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="55.5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:7" ht="54" x14ac:dyDescent="0.35">
       <c r="A1" s="22" t="s">
         <v>368</v>
       </c>
@@ -4318,7 +4322,7 @@
       <c r="F1" s="11"/>
       <c r="G1" s="11"/>
     </row>
-    <row r="2" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A2" s="23" t="s">
         <v>369</v>
       </c>
@@ -4329,7 +4333,7 @@
       <c r="F2" s="11"/>
       <c r="G2" s="11"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="12" t="s">
         <v>370</v>
       </c>
@@ -4352,7 +4356,7 @@
         <v>376</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="13" t="s">
         <v>377</v>
       </c>
@@ -4376,7 +4380,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="13" t="s">
         <v>377</v>
       </c>
@@ -4400,7 +4404,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="13" t="s">
         <v>388</v>
       </c>
@@ -4418,13 +4422,13 @@
       </c>
       <c r="F7" s="15">
         <f>RawMaterials!B8</f>
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="G7" s="13" t="s">
         <v>392</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="13" t="s">
         <v>388</v>
       </c>
@@ -4442,13 +4446,13 @@
       </c>
       <c r="F8" s="15">
         <f>RawMaterials!B21</f>
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="G8" s="13" t="s">
         <v>392</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="13" t="s">
         <v>397</v>
       </c>
@@ -4472,7 +4476,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A10" s="16" t="s">
         <v>403</v>
       </c>
@@ -4496,7 +4500,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="16" t="s">
         <v>403</v>
       </c>
@@ -4520,7 +4524,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="16" t="s">
         <v>414</v>
       </c>
@@ -4544,7 +4548,7 @@
         <v>418</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="13" t="s">
         <v>419</v>
       </c>
@@ -4568,7 +4572,7 @@
         <v>423</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" s="20"/>
       <c r="B14" s="20"/>
       <c r="C14" s="20"/>
@@ -4577,7 +4581,7 @@
       <c r="F14" s="20"/>
       <c r="G14" s="20"/>
     </row>
-    <row r="15" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A15" s="21" t="s">
         <v>424</v>
       </c>
@@ -4596,27 +4600,27 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{96BAAF9A-F941-44AB-AA34-B72802C7CB08}">
   <dimension ref="A1:F26"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="30.6328125" customWidth="1"/>
-    <col min="2" max="2" width="14.6328125" customWidth="1"/>
-    <col min="3" max="3" width="14.6328125" style="53" customWidth="1"/>
-    <col min="4" max="4" width="14.6328125" customWidth="1"/>
-    <col min="5" max="5" width="14.6328125" style="53" customWidth="1"/>
-    <col min="6" max="6" width="14.6328125" customWidth="1"/>
+    <col min="1" max="1" width="30.6640625" customWidth="1"/>
+    <col min="2" max="2" width="14.6640625" customWidth="1"/>
+    <col min="3" max="3" width="14.6640625" style="53" customWidth="1"/>
+    <col min="4" max="4" width="14.6640625" customWidth="1"/>
+    <col min="5" max="5" width="14.6640625" style="53" customWidth="1"/>
+    <col min="6" max="6" width="14.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>425</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>426</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="52" t="s">
         <v>142</v>
       </c>
@@ -4636,7 +4640,7 @@
         <v>429</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="str">
         <f>Capacity!A4</f>
         <v>Cut handle</v>
@@ -4662,7 +4666,7 @@
         <v>add 1 machine</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="str">
         <f>Capacity!A5</f>
         <v>Internal thread (middle)</v>
@@ -4688,7 +4692,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" t="str">
         <f>Capacity!A6</f>
         <v>Stamp / narrow end (grip)</v>
@@ -4714,7 +4718,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" t="str">
         <f>Capacity!A7</f>
         <v>Knurl + external thread (grip)</v>
@@ -4740,7 +4744,7 @@
         <v>add 1 machine</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" t="str">
         <f>Capacity!A8</f>
         <v>Stamp shovel head</v>
@@ -4766,7 +4770,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" t="str">
         <f>Capacity!A9</f>
         <v>Shape / bend head</v>
@@ -4792,7 +4796,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" t="str">
         <f>Capacity!A10</f>
         <v>Sharpen blade</v>
@@ -4818,7 +4822,7 @@
         <v>add 1 machine</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" t="str">
         <f>Capacity!A11</f>
         <v>Serrate edge</v>
@@ -4844,7 +4848,7 @@
         <v>add 1 machine</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" t="str">
         <f>Capacity!A12</f>
         <v>Stamp hinge connector</v>
@@ -4870,7 +4874,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" t="str">
         <f>Capacity!A13</f>
         <v>Bend hinge connector</v>
@@ -4896,7 +4900,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" t="str">
         <f>Capacity!A14</f>
         <v>Rivet hinge to head</v>
@@ -4922,7 +4926,7 @@
         <v/>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" t="str">
         <f>Capacity!A15</f>
         <v>Hand polish / deburr</v>
@@ -4948,7 +4952,7 @@
         <v>add 1 machine</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" t="str">
         <f>Capacity!A16</f>
         <v>Final assembly</v>
@@ -4974,7 +4978,7 @@
         <v>add 1 machine</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" t="str">
         <f>Capacity!A17</f>
         <v>Packaging (hand + check)</v>
@@ -5000,12 +5004,12 @@
         <v>add 1 machine</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>430</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>431</v>
       </c>
@@ -5013,7 +5017,7 @@
         <v>432</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>433</v>
       </c>
@@ -5021,7 +5025,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>435</v>
       </c>
@@ -5029,7 +5033,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>437</v>
       </c>
@@ -5037,7 +5041,7 @@
         <v>438</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>439</v>
       </c>
@@ -5053,21 +5057,21 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4BDF06B8-739A-4DCC-9B6F-2B6AC0031BE6}">
   <dimension ref="A1:E55"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="50.6328125" customWidth="1"/>
-    <col min="2" max="2" width="14.6328125" customWidth="1"/>
-    <col min="3" max="3" width="22.6328125" customWidth="1"/>
-    <col min="4" max="4" width="18.6328125" customWidth="1"/>
-    <col min="5" max="5" width="60.6328125" customWidth="1"/>
+    <col min="1" max="1" width="50.6640625" customWidth="1"/>
+    <col min="2" max="2" width="14.6640625" customWidth="1"/>
+    <col min="3" max="3" width="22.6640625" customWidth="1"/>
+    <col min="4" max="4" width="18.6640625" customWidth="1"/>
+    <col min="5" max="5" width="60.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>449</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="52" t="s">
         <v>450</v>
       </c>
@@ -5084,119 +5088,119 @@
         <v>453</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>454</v>
       </c>
       <c r="B4" s="56">
         <f>Space_Summary!B14-Space_Summary!B10-Space_Summary!B11-Space_Summary!B5</f>
-        <v>1077.4880000000001</v>
+        <v>957.59375</v>
       </c>
       <c r="C4" s="56">
         <v>8500</v>
       </c>
       <c r="D4" s="56">
         <f>B4*C4</f>
-        <v>9158648</v>
+        <v>8139546.875</v>
       </c>
       <c r="E4" t="s">
         <v>455</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>456</v>
       </c>
       <c r="B5" s="56">
         <f>Space_Summary!B10</f>
-        <v>260</v>
+        <v>216</v>
       </c>
       <c r="C5" s="56">
         <v>12000</v>
       </c>
       <c r="D5" s="56">
         <f>B5*C5</f>
-        <v>3120000</v>
+        <v>2592000</v>
       </c>
       <c r="E5" t="s">
         <v>457</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>458</v>
       </c>
       <c r="B6" s="56">
         <f>Space_Summary!B11</f>
-        <v>240</v>
+        <v>203</v>
       </c>
       <c r="C6" s="56">
         <v>10000</v>
       </c>
       <c r="D6" s="56">
         <f>B6*C6</f>
-        <v>2400000</v>
+        <v>2030000</v>
       </c>
       <c r="E6" t="s">
         <v>457</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>459</v>
       </c>
       <c r="B7" s="56">
         <f>Space_Summary!B5</f>
-        <v>120</v>
+        <v>135</v>
       </c>
       <c r="C7" s="56">
         <v>18000</v>
       </c>
       <c r="D7" s="56">
         <f>B7*C7</f>
-        <v>2160000</v>
+        <v>2430000</v>
       </c>
       <c r="E7" t="s">
         <v>460</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>461</v>
       </c>
       <c r="B8" s="56">
         <f>Parking!B10</f>
-        <v>2110</v>
+        <v>2198</v>
       </c>
       <c r="C8" s="56">
         <v>1200</v>
       </c>
       <c r="D8" s="56">
         <f>B8*C8</f>
-        <v>2532000</v>
+        <v>2637600</v>
       </c>
       <c r="E8" t="s">
         <v>457</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="52" t="s">
         <v>462</v>
       </c>
       <c r="D9" s="57">
         <f>SUM(D4:D8)</f>
-        <v>19370648</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+        <v>17829146.875</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="D10" s="56"/>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" s="52" t="s">
         <v>463</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" s="52" t="s">
         <v>464</v>
       </c>
@@ -5213,7 +5217,7 @@
         <v>467</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>557</v>
       </c>
@@ -5225,14 +5229,14 @@
         <v>350000</v>
       </c>
       <c r="D13" s="56">
-        <f>B13*C13</f>
+        <f t="shared" ref="D13:D31" si="0">B13*C13</f>
         <v>700000</v>
       </c>
       <c r="E13" t="s">
         <v>558</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>559</v>
       </c>
@@ -5244,14 +5248,14 @@
         <v>180000</v>
       </c>
       <c r="D14" s="56">
-        <f>B14*C14</f>
+        <f t="shared" si="0"/>
         <v>360000</v>
       </c>
       <c r="E14" t="s">
         <v>560</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>561</v>
       </c>
@@ -5263,14 +5267,14 @@
         <v>250000</v>
       </c>
       <c r="D15" s="56">
-        <f>B15*C15</f>
+        <f t="shared" si="0"/>
         <v>250000</v>
       </c>
       <c r="E15" t="s">
         <v>562</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>563</v>
       </c>
@@ -5282,14 +5286,14 @@
         <v>380000</v>
       </c>
       <c r="D16" s="56">
-        <f>B16*C16</f>
+        <f t="shared" si="0"/>
         <v>1520000</v>
       </c>
       <c r="E16" t="s">
         <v>564</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>565</v>
       </c>
@@ -5301,14 +5305,14 @@
         <v>450000</v>
       </c>
       <c r="D17" s="56">
-        <f>B17*C17</f>
+        <f t="shared" si="0"/>
         <v>450000</v>
       </c>
       <c r="E17" t="s">
         <v>566</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>567</v>
       </c>
@@ -5320,14 +5324,14 @@
         <v>300000</v>
       </c>
       <c r="D18" s="56">
-        <f>B18*C18</f>
+        <f t="shared" si="0"/>
         <v>300000</v>
       </c>
       <c r="E18" t="s">
         <v>568</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>569</v>
       </c>
@@ -5339,14 +5343,14 @@
         <v>280000</v>
       </c>
       <c r="D19" s="56">
-        <f>B19*C19</f>
+        <f t="shared" si="0"/>
         <v>2240000</v>
       </c>
       <c r="E19" t="s">
         <v>570</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>571</v>
       </c>
@@ -5358,14 +5362,14 @@
         <v>220000</v>
       </c>
       <c r="D20" s="56">
-        <f>B20*C20</f>
+        <f t="shared" si="0"/>
         <v>880000</v>
       </c>
       <c r="E20" t="s">
         <v>572</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>573</v>
       </c>
@@ -5377,14 +5381,14 @@
         <v>280000</v>
       </c>
       <c r="D21" s="56">
-        <f>B21*C21</f>
+        <f t="shared" si="0"/>
         <v>280000</v>
       </c>
       <c r="E21" t="s">
         <v>566</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>574</v>
       </c>
@@ -5396,14 +5400,14 @@
         <v>180000</v>
       </c>
       <c r="D22" s="56">
-        <f>B22*C22</f>
+        <f t="shared" si="0"/>
         <v>180000</v>
       </c>
       <c r="E22" t="s">
         <v>568</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>575</v>
       </c>
@@ -5415,14 +5419,14 @@
         <v>60000</v>
       </c>
       <c r="D23" s="56">
-        <f>B23*C23</f>
+        <f t="shared" si="0"/>
         <v>60000</v>
       </c>
       <c r="E23" t="s">
         <v>576</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>577</v>
       </c>
@@ -5434,14 +5438,14 @@
         <v>120000</v>
       </c>
       <c r="D24" s="56">
-        <f>B24*C24</f>
+        <f t="shared" si="0"/>
         <v>480000</v>
       </c>
       <c r="E24" t="s">
         <v>578</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>579</v>
       </c>
@@ -5453,14 +5457,14 @@
         <v>40000</v>
       </c>
       <c r="D25" s="56">
-        <f>B25*C25</f>
+        <f t="shared" si="0"/>
         <v>80000</v>
       </c>
       <c r="E25" t="s">
         <v>580</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>581</v>
       </c>
@@ -5472,14 +5476,14 @@
         <v>35000</v>
       </c>
       <c r="D26" s="56">
-        <f>B26*C26</f>
+        <f t="shared" si="0"/>
         <v>70000</v>
       </c>
       <c r="E26" t="s">
         <v>580</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>582</v>
       </c>
@@ -5491,14 +5495,14 @@
         <v>950000</v>
       </c>
       <c r="D27" s="56">
-        <f>B27*C27</f>
+        <f t="shared" si="0"/>
         <v>950000</v>
       </c>
       <c r="E27" t="s">
         <v>583</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>584</v>
       </c>
@@ -5509,14 +5513,14 @@
         <v>650000</v>
       </c>
       <c r="D28" s="56">
-        <f>B28*C28</f>
+        <f t="shared" si="0"/>
         <v>650000</v>
       </c>
       <c r="E28" t="s">
         <v>585</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>586</v>
       </c>
@@ -5528,14 +5532,14 @@
         <v>2800000</v>
       </c>
       <c r="D29" s="56">
-        <f>B29*C29</f>
+        <f t="shared" si="0"/>
         <v>5600000</v>
       </c>
       <c r="E29" t="s">
         <v>587</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>588</v>
       </c>
@@ -5546,14 +5550,14 @@
         <v>450000</v>
       </c>
       <c r="D30" s="56">
-        <f>B30*C30</f>
+        <f t="shared" si="0"/>
         <v>1350000</v>
       </c>
       <c r="E30" t="s">
         <v>589</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>590</v>
       </c>
@@ -5564,14 +5568,14 @@
         <v>18000</v>
       </c>
       <c r="D31" s="56">
-        <f>B31*C31</f>
+        <f t="shared" si="0"/>
         <v>144000</v>
       </c>
       <c r="E31" t="s">
         <v>591</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" s="52" t="s">
         <v>468</v>
       </c>
@@ -5580,21 +5584,21 @@
         <v>16544000</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" s="52" t="s">
         <v>592</v>
       </c>
       <c r="D34" s="58">
         <f>D9+D32</f>
-        <v>35914648</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+        <v>34373146.875</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36" s="52" t="s">
         <v>469</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A37" s="52" t="s">
         <v>470</v>
       </c>
@@ -5611,7 +5615,7 @@
         <v>474</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>593</v>
       </c>
@@ -5628,7 +5632,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>596</v>
       </c>
@@ -5645,7 +5649,7 @@
         <v>598</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>599</v>
       </c>
@@ -5662,7 +5666,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>601</v>
       </c>
@@ -5679,7 +5683,7 @@
         <v>602</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>603</v>
       </c>
@@ -5696,7 +5700,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>605</v>
       </c>
@@ -5713,7 +5717,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>608</v>
       </c>
@@ -5730,7 +5734,7 @@
         <v>609</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>610</v>
       </c>
@@ -5747,12 +5751,12 @@
         <v>611</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A47" s="52" t="s">
         <v>475</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A48" s="52" t="s">
         <v>476</v>
       </c>
@@ -5763,7 +5767,7 @@
         <v>478</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>612</v>
       </c>
@@ -5774,7 +5778,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>615</v>
       </c>
@@ -5785,7 +5789,7 @@
         <v>617</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>618</v>
       </c>
@@ -5796,7 +5800,7 @@
         <v>620</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>621</v>
       </c>
@@ -5807,7 +5811,7 @@
         <v>623</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>624</v>
       </c>
@@ -5818,7 +5822,7 @@
         <v>626</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>627</v>
       </c>
@@ -5829,7 +5833,7 @@
         <v>629</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>630</v>
       </c>
@@ -5848,29 +5852,29 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F3CFA77-F31D-4AAF-BF8B-1DD55A6DB9DF}">
   <dimension ref="A1:G19"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="6.6328125" customWidth="1"/>
-    <col min="2" max="2" width="42.6328125" customWidth="1"/>
-    <col min="3" max="3" width="50.6328125" customWidth="1"/>
-    <col min="4" max="4" width="16.6328125" customWidth="1"/>
-    <col min="5" max="5" width="14.6328125" customWidth="1"/>
-    <col min="6" max="6" width="38.6328125" customWidth="1"/>
-    <col min="7" max="7" width="14.6328125" customWidth="1"/>
+    <col min="1" max="1" width="6.6640625" customWidth="1"/>
+    <col min="2" max="2" width="42.6640625" customWidth="1"/>
+    <col min="3" max="3" width="50.6640625" customWidth="1"/>
+    <col min="4" max="4" width="16.6640625" customWidth="1"/>
+    <col min="5" max="5" width="14.6640625" customWidth="1"/>
+    <col min="6" max="6" width="38.6640625" customWidth="1"/>
+    <col min="7" max="7" width="14.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="11" customFormat="1" ht="217.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" s="11" customFormat="1" ht="216" x14ac:dyDescent="0.3">
       <c r="A1" s="11" t="s">
         <v>479</v>
       </c>
     </row>
-    <row r="2" spans="1:7" s="11" customFormat="1" ht="304.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" s="11" customFormat="1" ht="302.39999999999998" x14ac:dyDescent="0.3">
       <c r="A2" s="11" t="s">
         <v>488</v>
       </c>
     </row>
-    <row r="3" spans="1:7" s="11" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="4" spans="1:7" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" s="11" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="4" spans="1:7" s="11" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A4" s="59" t="s">
         <v>480</v>
       </c>
@@ -5893,7 +5897,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="5" spans="1:7" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" s="11" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A5" s="11" t="s">
         <v>489</v>
       </c>
@@ -5917,7 +5921,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="6" spans="1:7" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" s="11" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A6" s="11" t="s">
         <v>495</v>
       </c>
@@ -5941,7 +5945,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="7" spans="1:7" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" s="11" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A7" s="11" t="s">
         <v>499</v>
       </c>
@@ -5965,7 +5969,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="8" spans="1:7" s="11" customFormat="1" ht="29" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" s="11" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" s="11" t="s">
         <v>503</v>
       </c>
@@ -5977,7 +5981,7 @@
       </c>
       <c r="D8" s="11">
         <f>Space_Summary!B5</f>
-        <v>120</v>
+        <v>135</v>
       </c>
       <c r="E8" s="11" t="s">
         <v>506</v>
@@ -5989,7 +5993,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="9" spans="1:7" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:7" s="11" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9" s="11" t="s">
         <v>508</v>
       </c>
@@ -6013,7 +6017,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="10" spans="1:7" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:7" s="11" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A10" s="11" t="s">
         <v>513</v>
       </c>
@@ -6037,7 +6041,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="11" spans="1:7" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:7" s="11" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A11" s="11" t="s">
         <v>517</v>
       </c>
@@ -6049,7 +6053,7 @@
       </c>
       <c r="D11" s="11">
         <f>Space_Summary!B15</f>
-        <v>170</v>
+        <v>151</v>
       </c>
       <c r="E11" s="11" t="s">
         <v>520</v>
@@ -6061,7 +6065,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="12" spans="1:7" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:7" s="11" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A12" s="11" t="s">
         <v>522</v>
       </c>
@@ -6085,7 +6089,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="13" spans="1:7" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:7" s="11" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A13" s="11" t="s">
         <v>527</v>
       </c>
@@ -6097,7 +6101,7 @@
       </c>
       <c r="D13" s="11">
         <f>Parking!B8</f>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E13" s="11" t="s">
         <v>525</v>
@@ -6109,7 +6113,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="14" spans="1:7" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:7" s="11" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A14" s="11" t="s">
         <v>531</v>
       </c>
@@ -6121,7 +6125,7 @@
       </c>
       <c r="D14" s="11">
         <f>Space_Summary!B6</f>
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="E14" s="11">
         <v>6.5</v>
@@ -6133,7 +6137,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="15" spans="1:7" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:7" s="11" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A15" s="11" t="s">
         <v>535</v>
       </c>
@@ -6145,7 +6149,7 @@
       </c>
       <c r="D15" s="11">
         <f>Evaluation!F11</f>
-        <v>4.45</v>
+        <v>4.1000000000000005</v>
       </c>
       <c r="E15" s="11" t="s">
         <v>538</v>
@@ -6157,7 +6161,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="16" spans="1:7" s="11" customFormat="1" ht="29" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:7" s="11" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A16" s="11" t="s">
         <v>540</v>
       </c>
@@ -6169,7 +6173,7 @@
       </c>
       <c r="D16" s="11">
         <f>Space_Summary!B16</f>
-        <v>1867</v>
+        <v>1663</v>
       </c>
       <c r="E16" s="11">
         <v>9</v>
@@ -6181,7 +6185,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="17" spans="1:7" s="11" customFormat="1" ht="29" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:7" s="11" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A17" s="11" t="s">
         <v>544</v>
       </c>
@@ -6193,7 +6197,7 @@
       </c>
       <c r="D17" s="11">
         <f>Personnel!B18</f>
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E17" s="11" t="s">
         <v>525</v>
@@ -6205,7 +6209,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="18" spans="1:7" s="11" customFormat="1" ht="29" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:7" s="11" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A18" s="11" t="s">
         <v>548</v>
       </c>
@@ -6228,7 +6232,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="19" spans="1:7" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:7" s="11" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A19" s="11" t="s">
         <v>552</v>
       </c>
@@ -6259,15 +6263,15 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:D17"/>
-  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="40.1796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.6328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.6328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="40.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="17" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A1" s="27" t="s">
         <v>121</v>
       </c>
@@ -6275,13 +6279,13 @@
       <c r="C1" s="27"/>
       <c r="D1" s="27"/>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="25"/>
       <c r="B2" s="25"/>
       <c r="C2" s="25"/>
       <c r="D2" s="25"/>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="28" t="s">
         <v>122</v>
       </c>
@@ -6295,7 +6299,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="24" t="s">
         <v>5</v>
       </c>
@@ -6310,7 +6314,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="24" t="s">
         <v>125</v>
       </c>
@@ -6325,7 +6329,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="24" t="s">
         <v>10</v>
       </c>
@@ -6340,7 +6344,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="24" t="s">
         <v>18</v>
       </c>
@@ -6355,7 +6359,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="24" t="s">
         <v>127</v>
       </c>
@@ -6370,7 +6374,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="24" t="s">
         <v>26</v>
       </c>
@@ -6385,13 +6389,13 @@
         <v>130</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" s="25"/>
       <c r="B10" s="25"/>
       <c r="C10" s="25"/>
       <c r="D10" s="25"/>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" s="29" t="s">
         <v>131</v>
       </c>
@@ -6399,7 +6403,7 @@
       <c r="C11" s="29"/>
       <c r="D11" s="29"/>
     </row>
-    <row r="12" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A12" s="28" t="s">
         <v>132</v>
       </c>
@@ -6413,7 +6417,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" s="25" t="s">
         <v>136</v>
       </c>
@@ -6426,7 +6430,7 @@
       </c>
       <c r="D13" s="25"/>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" s="25" t="s">
         <v>137</v>
       </c>
@@ -6439,7 +6443,7 @@
       </c>
       <c r="D14" s="25"/>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" s="25" t="s">
         <v>138</v>
       </c>
@@ -6455,7 +6459,7 @@
         <v>3829.4736842105267</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" s="25" t="s">
         <v>139</v>
       </c>
@@ -6471,7 +6475,7 @@
         <v>1914.7368421052633</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" s="25" t="s">
         <v>140</v>
       </c>
@@ -6496,25 +6500,25 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:P19"/>
-  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="48.90625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.36328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="48.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.33203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="7" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.5546875" bestFit="1" customWidth="1"/>
     <col min="5" max="7" width="12" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="6.1796875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="6.21875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="12" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="8" customWidth="1"/>
     <col min="11" max="11" width="12" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.6328125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.36328125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.33203125" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="6" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="8.54296875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="64.90625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="8.5546875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="64.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="17" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:16" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A1" s="27" t="s">
         <v>141</v>
       </c>
@@ -6534,7 +6538,7 @@
       <c r="O1" s="27"/>
       <c r="P1" s="27"/>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A2" s="25"/>
       <c r="B2" s="25"/>
       <c r="C2" s="25"/>
@@ -6552,7 +6556,7 @@
       <c r="O2" s="25"/>
       <c r="P2" s="25"/>
     </row>
-    <row r="3" spans="1:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:16" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A3" s="28" t="s">
         <v>142</v>
       </c>
@@ -6602,7 +6606,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A4" s="30" t="s">
         <v>157</v>
       </c>
@@ -6662,7 +6666,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A5" s="25" t="s">
         <v>161</v>
       </c>
@@ -6721,7 +6725,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A6" s="30" t="s">
         <v>165</v>
       </c>
@@ -6780,7 +6784,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A7" s="25" t="s">
         <v>166</v>
       </c>
@@ -6839,7 +6843,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A8" s="30" t="s">
         <v>167</v>
       </c>
@@ -6898,7 +6902,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A9" s="25" t="s">
         <v>170</v>
       </c>
@@ -6957,7 +6961,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A10" s="30" t="s">
         <v>172</v>
       </c>
@@ -7016,7 +7020,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A11" s="25" t="s">
         <v>175</v>
       </c>
@@ -7075,7 +7079,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A12" s="30" t="s">
         <v>176</v>
       </c>
@@ -7134,7 +7138,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A13" s="25" t="s">
         <v>177</v>
       </c>
@@ -7193,7 +7197,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A14" s="30" t="s">
         <v>178</v>
       </c>
@@ -7252,7 +7256,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A15" s="25" t="s">
         <v>179</v>
       </c>
@@ -7311,7 +7315,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A16" s="30" t="s">
         <v>180</v>
       </c>
@@ -7370,7 +7374,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="17" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="35" t="s">
         <v>181</v>
       </c>
@@ -7430,7 +7434,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="18" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A18" s="41" t="s">
         <v>183</v>
       </c>
@@ -7456,7 +7460,7 @@
       </c>
       <c r="P18" s="41"/>
     </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A19" s="40" t="s">
         <v>364</v>
       </c>
@@ -7488,38 +7492,38 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:C20"/>
-  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="74.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="74.77734375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="6" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.08984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="17" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A1" s="27" t="s">
         <v>184</v>
       </c>
       <c r="B1" s="27"/>
       <c r="C1" s="27"/>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="25"/>
       <c r="B2" s="25"/>
       <c r="C2" s="25"/>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="29" t="s">
         <v>185</v>
       </c>
       <c r="B3" s="29"/>
       <c r="C3" s="29"/>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="25"/>
       <c r="B4" s="25"/>
       <c r="C4" s="25"/>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="24" t="s">
         <v>186</v>
       </c>
@@ -7531,7 +7535,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="24" t="s">
         <v>188</v>
       </c>
@@ -7543,7 +7547,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="24" t="s">
         <v>189</v>
       </c>
@@ -7555,7 +7559,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="24" t="s">
         <v>191</v>
       </c>
@@ -7567,7 +7571,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="24" t="s">
         <v>192</v>
       </c>
@@ -7579,26 +7583,26 @@
         <v>193</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" s="26" t="s">
         <v>194</v>
       </c>
       <c r="B10" s="25"/>
       <c r="C10" s="25"/>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="25"/>
       <c r="B11" s="25"/>
       <c r="C11" s="25"/>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" s="29" t="s">
         <v>195</v>
       </c>
       <c r="B12" s="29"/>
       <c r="C12" s="29"/>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" s="24" t="s">
         <v>196</v>
       </c>
@@ -7610,7 +7614,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" s="24" t="s">
         <v>197</v>
       </c>
@@ -7622,7 +7626,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" s="24" t="s">
         <v>199</v>
       </c>
@@ -7633,26 +7637,26 @@
         <v>200</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" s="26" t="s">
         <v>201</v>
       </c>
       <c r="B16" s="25"/>
       <c r="C16" s="25"/>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" s="25"/>
       <c r="B17" s="25"/>
       <c r="C17" s="25"/>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" s="29" t="s">
         <v>202</v>
       </c>
       <c r="B18" s="29"/>
       <c r="C18" s="29"/>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" s="24" t="s">
         <v>203</v>
       </c>
@@ -7664,7 +7668,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" s="26" t="s">
         <v>204</v>
       </c>
@@ -7680,33 +7684,33 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:C22"/>
-  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="29.36328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.36328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="29.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="17" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A1" s="27" t="s">
         <v>205</v>
       </c>
       <c r="B1" s="27"/>
       <c r="C1" s="27"/>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="25"/>
       <c r="B2" s="25"/>
       <c r="C2" s="25"/>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="29" t="s">
         <v>206</v>
       </c>
       <c r="B3" s="29"/>
       <c r="C3" s="29"/>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="24" t="s">
         <v>207</v>
       </c>
@@ -7718,7 +7722,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="24" t="s">
         <v>208</v>
       </c>
@@ -7730,7 +7734,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="24" t="s">
         <v>210</v>
       </c>
@@ -7742,55 +7746,55 @@
         <v>209</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="24" t="s">
         <v>211</v>
       </c>
       <c r="B7" s="48">
         <f>Inputs!$C$21</f>
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C7" s="25" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="24" t="s">
         <v>212</v>
       </c>
       <c r="B8" s="49">
         <f>ROUNDUP(B6/B7,0)</f>
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="C8" s="25" t="s">
         <v>213</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="24" t="s">
         <v>214</v>
       </c>
       <c r="B9" s="49">
         <f>B8*Inputs!$C$30</f>
-        <v>960</v>
+        <v>900</v>
       </c>
       <c r="C9" s="25" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" s="25"/>
       <c r="B10" s="48"/>
       <c r="C10" s="25"/>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="29" t="s">
         <v>215</v>
       </c>
       <c r="B11" s="50"/>
       <c r="C11" s="29"/>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" s="24" t="s">
         <v>216</v>
       </c>
@@ -7802,7 +7806,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" s="24" t="s">
         <v>217</v>
       </c>
@@ -7814,7 +7818,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" s="24" t="s">
         <v>218</v>
       </c>
@@ -7826,31 +7830,31 @@
         <v>78</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" s="24" t="s">
         <v>219</v>
       </c>
       <c r="B15" s="48">
         <f>FLOOR(B12*Inputs!$C$25/B13,1)</f>
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="C15" s="25" t="s">
         <v>220</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" s="24" t="s">
         <v>221</v>
       </c>
       <c r="B16" s="48">
         <f>FLOOR(B12*Inputs!$C$25/B14,1)</f>
-        <v>585</v>
+        <v>625</v>
       </c>
       <c r="C16" s="25" t="s">
         <v>220</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" s="24" t="s">
         <v>222</v>
       </c>
@@ -7862,7 +7866,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" s="24" t="s">
         <v>224</v>
       </c>
@@ -7874,19 +7878,19 @@
         <v>223</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" s="24" t="s">
         <v>225</v>
       </c>
       <c r="B19" s="48">
         <f>ROUNDUP(B17/B15,0)</f>
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C19" s="25" t="s">
         <v>226</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A20" s="36" t="s">
         <v>227</v>
       </c>
@@ -7898,25 +7902,25 @@
         <v>226</v>
       </c>
     </row>
-    <row r="21" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A21" s="41" t="s">
         <v>228</v>
       </c>
       <c r="B21" s="41">
         <f>B19+B20</f>
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C21" s="41" t="s">
         <v>226</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" s="40" t="s">
         <v>229</v>
       </c>
       <c r="B22" s="40">
         <f>B21*Inputs!$C$30</f>
-        <v>240</v>
+        <v>230</v>
       </c>
       <c r="C22" s="40" t="s">
         <v>85</v>
@@ -7931,33 +7935,33 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:C15"/>
-  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="43.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="43.77734375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="6" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.90625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="17" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A1" s="27" t="s">
         <v>230</v>
       </c>
       <c r="B1" s="27"/>
       <c r="C1" s="27"/>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="25"/>
       <c r="B2" s="25"/>
       <c r="C2" s="25"/>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="29" t="s">
         <v>231</v>
       </c>
       <c r="B3" s="29"/>
       <c r="C3" s="29"/>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="24" t="s">
         <v>232</v>
       </c>
@@ -7969,7 +7973,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="24" t="s">
         <v>233</v>
       </c>
@@ -7981,7 +7985,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="24" t="s">
         <v>234</v>
       </c>
@@ -7993,91 +7997,91 @@
         <v>69</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="25"/>
       <c r="B7" s="25"/>
       <c r="C7" s="25"/>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="29" t="s">
         <v>235</v>
       </c>
       <c r="B8" s="29"/>
       <c r="C8" s="29"/>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="24" t="s">
         <v>68</v>
       </c>
       <c r="B9" s="25">
         <f>Inputs!$C$33</f>
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C9" s="25" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" s="24" t="s">
         <v>70</v>
       </c>
       <c r="B10" s="25">
         <f>Inputs!$C$34</f>
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="C10" s="25" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="24" t="s">
         <v>72</v>
       </c>
       <c r="B11" s="25">
         <f>Inputs!$C$35</f>
-        <v>400</v>
+        <v>360</v>
       </c>
       <c r="C11" s="25" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" s="24" t="s">
         <v>236</v>
       </c>
       <c r="B12" s="25">
         <f>ROUNDUP(Inputs!$C$7/Inputs!$C$33,0)</f>
-        <v>182</v>
+        <v>228</v>
       </c>
       <c r="C12" s="25" t="s">
         <v>237</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" s="24" t="s">
         <v>238</v>
       </c>
       <c r="B13" s="24">
         <f>ROUNDUP(Inputs!$C$7/Inputs!$C$35,0)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C13" s="25" t="s">
         <v>239</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" s="24" t="s">
         <v>240</v>
       </c>
       <c r="B14" s="25">
         <f>Inputs!$C$35</f>
-        <v>400</v>
+        <v>360</v>
       </c>
       <c r="C14" s="25" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" s="24" t="s">
         <v>242</v>
       </c>
@@ -8097,16 +8101,16 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:E9"/>
-  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="30.1796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="5.6328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.36328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.90625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.6328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="30.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.88671875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="17" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A1" s="27" t="s">
         <v>243</v>
       </c>
@@ -8115,14 +8119,14 @@
       <c r="D1" s="27"/>
       <c r="E1" s="27"/>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="25"/>
       <c r="B2" s="25"/>
       <c r="C2" s="25"/>
       <c r="D2" s="25"/>
       <c r="E2" s="25"/>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="28" t="s">
         <v>244</v>
       </c>
@@ -8139,33 +8143,33 @@
         <v>123</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="24" t="s">
         <v>248</v>
       </c>
       <c r="B4" s="25">
         <f>RawMaterials!B9</f>
-        <v>960</v>
+        <v>900</v>
       </c>
       <c r="C4" s="25">
         <f>ROUNDUP(RawMaterials!B9/Inputs!$C$40,0)</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D4" s="24">
         <f>C4*Inputs!$C$41*Inputs!$C$43</f>
-        <v>38.400000000000006</v>
+        <v>37.5</v>
       </c>
       <c r="E4" s="26" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="24" t="s">
         <v>250</v>
       </c>
       <c r="B5" s="25">
         <f>RawMaterials!B22</f>
-        <v>240</v>
+        <v>230</v>
       </c>
       <c r="C5" s="25">
         <f>ROUNDUP(RawMaterials!B22/Inputs!$C$42,0)</f>
@@ -8173,39 +8177,39 @@
       </c>
       <c r="D5" s="24">
         <f>C5*(Inputs!$C$23*Inputs!$C$24)*Inputs!$C$43</f>
-        <v>10</v>
+        <v>9.375</v>
       </c>
       <c r="E5" s="26" t="s">
         <v>251</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="24" t="s">
         <v>252</v>
       </c>
       <c r="B6" s="25">
         <f>ROUNDUP(Inventory_Pack!B5/Inputs!$C$35,0)</f>
-        <v>91</v>
+        <v>102</v>
       </c>
       <c r="C6" s="25">
         <f>ROUNDUP(B6/Inputs!$C$39,0)</f>
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="D6" s="24">
         <f>C6*Inputs!$C$38*Inputs!$C$43</f>
-        <v>59.519999999999996</v>
+        <v>46.8</v>
       </c>
       <c r="E6" s="26" t="s">
         <v>253</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="24" t="s">
         <v>254</v>
       </c>
       <c r="B7" s="25">
         <f>ROUNDUP(Inventory_Pack!B6/Inputs!$C$35,0)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C7" s="25">
         <f>ROUNDUP(B7/Inputs!$C$39,0)</f>
@@ -8213,13 +8217,13 @@
       </c>
       <c r="D7" s="24">
         <f>C7*Inputs!$C$38*Inputs!$C$43</f>
-        <v>3.84</v>
+        <v>3.5999999999999996</v>
       </c>
       <c r="E7" s="26" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="36" t="s">
         <v>256</v>
       </c>
@@ -8231,13 +8235,13 @@
       </c>
       <c r="D8" s="36">
         <f>Inputs!$C$52</f>
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="E8" s="38" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="40" t="s">
         <v>257</v>
       </c>
@@ -8245,7 +8249,7 @@
       <c r="C9" s="40"/>
       <c r="D9" s="40">
         <f>SUM(D4:D8)</f>
-        <v>151.76</v>
+        <v>127.27499999999999</v>
       </c>
       <c r="E9" s="40"/>
     </row>
@@ -8258,26 +8262,26 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:C18"/>
-  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="31.90625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.90625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="41.08984375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="31.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="41.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="17" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A1" s="27" t="s">
         <v>258</v>
       </c>
       <c r="B1" s="27"/>
       <c r="C1" s="27"/>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="25"/>
       <c r="B2" s="25"/>
       <c r="C2" s="25"/>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="28" t="s">
         <v>259</v>
       </c>
@@ -8288,7 +8292,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="25" t="s">
         <v>261</v>
       </c>
@@ -8299,7 +8303,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="25" t="s">
         <v>262</v>
       </c>
@@ -8310,7 +8314,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="25" t="s">
         <v>263</v>
       </c>
@@ -8321,7 +8325,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="25" t="s">
         <v>264</v>
       </c>
@@ -8332,7 +8336,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="25" t="s">
         <v>265</v>
       </c>
@@ -8343,7 +8347,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="25" t="s">
         <v>266</v>
       </c>
@@ -8354,7 +8358,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" s="25" t="s">
         <v>268</v>
       </c>
@@ -8365,7 +8369,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="25" t="s">
         <v>269</v>
       </c>
@@ -8376,7 +8380,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" s="25" t="s">
         <v>270</v>
       </c>
@@ -8387,51 +8391,51 @@
         <v>124</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" s="25" t="s">
         <v>271</v>
       </c>
       <c r="B13" s="25">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C13" s="26" t="s">
         <v>272</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" s="25" t="s">
         <v>273</v>
       </c>
       <c r="B14" s="25">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C14" s="26" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" s="25" t="s">
         <v>274</v>
       </c>
       <c r="B15" s="25">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C15" s="26" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" s="25" t="s">
         <v>275</v>
       </c>
       <c r="B16" s="25">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C16" s="26" t="s">
         <v>276</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="35" t="s">
         <v>277</v>
       </c>
@@ -8443,13 +8447,13 @@
         <v>278</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" s="40" t="s">
         <v>279</v>
       </c>
       <c r="B18" s="40">
         <f>SUM(B4:B17)</f>
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C18" s="40"/>
     </row>
@@ -8462,116 +8466,116 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:C10"/>
-  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="35.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="35.5546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="17" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A1" s="27" t="s">
         <v>280</v>
       </c>
       <c r="B1" s="27"/>
       <c r="C1" s="27"/>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="25"/>
       <c r="B2" s="25"/>
       <c r="C2" s="25"/>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="24" t="s">
         <v>281</v>
       </c>
       <c r="B3" s="25">
         <f>Personnel!B18</f>
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C3" s="25" t="s">
         <v>282</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="24" t="s">
         <v>283</v>
       </c>
       <c r="B4" s="25">
         <f>B3*Inputs!$C$56</f>
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C4" s="25" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="36" t="s">
         <v>113</v>
       </c>
       <c r="B5" s="35">
         <f>Inputs!$C$57</f>
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C5" s="35" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="40" t="s">
         <v>284</v>
       </c>
       <c r="B6" s="40">
         <f>B4+B5</f>
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C6" s="40" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="43" t="s">
         <v>285</v>
       </c>
       <c r="B7" s="43">
         <f>B6*Inputs!$C$58</f>
-        <v>1750</v>
+        <v>1848</v>
       </c>
       <c r="C7" s="39" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="24" t="s">
         <v>117</v>
       </c>
       <c r="B8" s="25">
         <f>Inputs!$C$59</f>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C8" s="25" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="36" t="s">
         <v>286</v>
       </c>
       <c r="B9" s="36">
         <f>B8*Inputs!$C$60</f>
-        <v>360</v>
+        <v>350</v>
       </c>
       <c r="C9" s="35" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" s="40" t="s">
         <v>287</v>
       </c>
       <c r="B10" s="40">
         <f>B7+B9</f>
-        <v>2110</v>
+        <v>2198</v>
       </c>
       <c r="C10" s="40" t="s">
         <v>78</v>

</xml_diff>